<commit_message>
Rebuild sheet template with confirmed hours; record handoff state
- Regenerate Flora_Booking_Sheet_Template.xlsx so Settings carries
  Monday–Sunday 7:30 AM–8:30 PM and the 8:30 PM return deadline.
- CLAUDE.md / AGENTS.md: repo now on GitHub, all sizes confirmed,
  remaining owner items, clasp setup status and TLS-inspection note,
  policy pop-up browser check, archive-tab workflow not yet built.
- OWNER_SETTINGS.md: template regenerated; Hibiscus size no longer open.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XCwLhjmsPGXo1UQCWYYhTX
</commit_message>
<xml_diff>
--- a/sheets-template/Flora_Booking_Sheet_Template.xlsx
+++ b/sheets-template/Flora_Booking_Sheet_Template.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Catalog" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Bookings" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Booking Items" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Blocked Dates" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Settings" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Catalog" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bookings" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Booking Items" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Blocked Dates" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Settings" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -543,7 +543,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Small</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -623,6 +623,11 @@
           <t>Beige lace midi dress with thin straps, a boned straight neckline and a soft A-line skirt.</t>
         </is>
       </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Small</t>
+        </is>
+      </c>
       <c r="E4" t="inlineStr">
         <is>
           <t>Beige</t>
@@ -779,7 +784,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Dusty blue-grey strapless corset mini dress with grey 3D flower appliquÃ©s, beading and a gathered bubble skirt.</t>
+          <t>Dusty blue-grey strapless corset mini dress with grey 3D flower appliqués, beading and a gathered bubble skirt.</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -13301,10 +13306,14 @@
           <t>operating_hours</t>
         </is>
       </c>
-      <c r="B5" s="3" t="n"/>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Monday–Sunday, 7:30 AM–8:30 PM</t>
+        </is>
+      </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>REQUIRED. Example: "Daily, 10:00 AM â€“ 6:00 PM".</t>
+          <t>Owner-confirmed hours. Pickup slots and return deadline are separate settings.</t>
         </is>
       </c>
     </row>
@@ -13327,10 +13336,14 @@
           <t>return_deadline_time</t>
         </is>
       </c>
-      <c r="B7" s="3" t="n"/>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>8:30 PM</t>
+        </is>
+      </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>REQUIRED. Time the dress is due back on the return date, e.g. 6:00 PM.</t>
+          <t>Owner-confirmed deadline on the return date (Asia/Manila).</t>
         </is>
       </c>
     </row>
@@ -13381,7 +13394,7 @@
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>Default â‚± per extra day (Catalog "Extension rate" overrides per dress).</t>
+          <t>Default ₱ per extra day (Catalog "Extension rate" overrides per dress).</t>
         </is>
       </c>
     </row>
@@ -13398,7 +13411,7 @@
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>per_dress: each dress pays â‚±100 per extra day (owner confirmed 2026-10-22).</t>
+          <t>per_dress: each dress pays ₱100 per extra day (owner confirmed 2026-10-22).</t>
         </is>
       </c>
     </row>
@@ -13449,7 +13462,7 @@
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>Refundable reservation/security deposit (â‚±). Separate from rental fees; never rental revenue.</t>
+          <t>Refundable reservation/security deposit (₱). Separate from rental fees; never rental revenue.</t>
         </is>
       </c>
     </row>
@@ -13466,7 +13479,7 @@
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>per_dress: â‚±500 refundable deposit for each dress (owner confirmed 2026-10-22).</t>
+          <t>per_dress: ₱500 refundable deposit for each dress (owner confirmed 2026-10-22).</t>
         </is>
       </c>
     </row>
@@ -13534,7 +13547,7 @@
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>Late return without an approved extension (â‚± per day). Shown in the terms.</t>
+          <t>Late return without an approved extension (₱ per day). Shown in the terms.</t>
         </is>
       </c>
     </row>
@@ -13547,27 +13560,27 @@
       <c r="B20" s="3" t="inlineStr">
         <is>
           <t>STANDARD RENTAL
-â€¢ The standard rental covers 3 calendar days, including pickup and return days: Day 1 pick up, Day 2 wear, Day 3 return.
-â€¢ Need 4 days? Add â‚±100 per dress. Further extensions cost â‚±100 per dress per extra day, subject to availability and prior approval.
-â€¢ Your exact pickup and return schedule is written in your rental agreement.
+• The standard rental covers 3 calendar days, including pickup and return days: Day 1 pick up, Day 2 wear, Day 3 return.
+• Need 4 days? Add ₱100 per dress. Further extensions cost ₱100 per dress per extra day, subject to availability and prior approval.
+• Your exact pickup and return schedule is written in your rental agreement.
 RESERVATION AND DEPOSIT
-â€¢ A â‚±500 refundable reservation/security deposit per dress secures your dress and dates. It is separate from the rental fee.
-â€¢ Please message us from an active, real Facebook account. We use it to verify your booking.
-â€¢ Your booking is confirmed only after we verify your payment and send confirmation.
-â€¢ The deposit is refunded after the dress is returned and inspected, less any documented charges under your rental agreement.
+• A ₱500 refundable reservation/security deposit per dress secures your dress and dates. It is separate from the rental fee.
+• Please message us from an active, real Facebook account. We use it to verify your booking.
+• Your booking is confirmed only after we verify your payment and send confirmation.
+• The deposit is refunded after the dress is returned and inspected, less any documented charges under your rental agreement.
 PICKUP
-â€¢ Present a valid government-issued photo ID, sign the rental agreement, and settle your rental fee. Your original ID is returned after verification.
-â€¢ We check the dress and included accessories with you before release.
+• Present a valid government-issued photo ID, sign the rental agreement, and settle your rental fee. Your original ID is returned after verification.
+• We check the dress and included accessories with you before release.
 CARE
-â€¢ Avoid makeup stains, food spills, and spraying perfume directly on the fabric.
-â€¢ Keep the dress away from sharp objects and rough surfaces.
-â€¢ Do not wash, dry-clean, iron, steam, pin, or alter the dress.
-â€¢ Ask for approval before using it in seawater, pools, or wet locations.
-â€¢ Report any damage or concerns immediately. Regular cleaning is included.
+• Avoid makeup stains, food spills, and spraying perfume directly on the fabric.
+• Keep the dress away from sharp objects and rough surfaces.
+• Do not wash, dry-clean, iron, steam, pin, or alter the dress.
+• Ask for approval before using it in seawater, pools, or wet locations.
+• Report any damage or concerns immediately. Regular cleaning is included.
 RETURN AND INSPECTION
-â€¢ Return the dress and all included accessories by the agreed date and time. Message us early if you expect a delay; an extension is only confirmed once approved.
-â€¢ Late return without an approved extension: â‚±120 per day.
-â€¢ We inspect the dress against its recorded pickup condition. Normal wear is not treated as damage. Extra cleaning, repairs, missing accessories, or loss may result in documented charges under your signed agreement.</t>
+• Return the dress and all included accessories by the agreed date and time. Message us early if you expect a delay; an extension is only confirmed once approved.
+• Late return without an approved extension: ₱120 per day.
+• We inspect the dress against its recorded pickup condition. Normal wear is not treated as damage. Extra cleaning, repairs, missing accessories, or loss may result in documented charges under your signed agreement.</t>
         </is>
       </c>
       <c r="C20" s="4" t="inlineStr">
@@ -13599,27 +13612,27 @@
         <is>
           <t>CANCELLATION AND REFUND POLICY
 Before your booking is confirmed
-â€¢ Sending a reservation request is free. If you change your mind before paying the deposit, just let us know or let the hold expire. Nothing is charged.
+• Sending a reservation request is free. If you change your mind before paying the deposit, just let us know or let the hold expire. Nothing is charged.
 If you cancel after your booking is confirmed
-The â‚±500 refundable security deposit (per dress) is handled as follows, counted from your pickup date:
-â€¢ 7 or more days before pickup: full deposit refunded.
-â€¢ 3 to 6 days before pickup: 50% of the deposit refunded, or move the full deposit to a new date within 60 days (once, subject to availability).
-â€¢ Less than 3 days before pickup, or no-show on pickup day: deposit forfeited.
-â€¢ The rental fee is paid at pickup, so there is nothing else to refund before pickup.
+The ₱500 refundable security deposit (per dress) is handled as follows, counted from your pickup date:
+• 7 or more days before pickup: full deposit refunded.
+• 3 to 6 days before pickup: 50% of the deposit refunded, or move the full deposit to a new date within 60 days (once, subject to availability).
+• Less than 3 days before pickup, or no-show on pickup day: deposit forfeited.
+• The rental fee is paid at pickup, so there is nothing else to refund before pickup.
 Changing your dates
-â€¢ You can move your booking once, free of charge, if you ask at least 3 days before pickup and the dress is available on the new dates.
-â€¢ Any price difference for extra days is settled at pickup.
+• You can move your booking once, free of charge, if you ask at least 3 days before pickup and the dress is available on the new dates.
+• Any price difference for extra days is settled at pickup.
 If Flora cancels
-â€¢ If we cannot provide your dress (for example, it is damaged or unavailable), you can choose another available dress for the same dates or a full refund of everything you have paid.
+• If we cannot provide your dress (for example, it is damaged or unavailable), you can choose another available dress for the same dates or a full refund of everything you have paid.
 Weather and emergencies
-â€¢ If PAGASA raises a Tropical Cyclone Wind Signal No. 2 or higher over Bohol, or the local government suspends activities on your pickup or event date, you may move your booking for free or get a full deposit refund.
+• If PAGASA raises a Tropical Cyclone Wind Signal No. 2 or higher over Bohol, or the local government suspends activities on your pickup or event date, you may move your booking for free or get a full deposit refund.
 After your rental
-â€¢ Returning the dress early does not reduce the rental fee.
-â€¢ Your deposit is refunded after the dress and accessories are returned and inspected, less any documented charges under your signed rental agreement (for example: late return at â‚±120 per day, extra cleaning, repairs, or missing items).
-â€¢ We explain every deduction with photos before releasing the balance.
+• Returning the dress early does not reduce the rental fee.
+• Your deposit is refunded after the dress and accessories are returned and inspected, less any documented charges under your signed rental agreement (for example: late return at ₱120 per day, extra cleaning, repairs, or missing items).
+• We explain every deduction with photos before releasing the balance.
 How refunds are paid
-â€¢ Refunds are sent within 3 business days after return and inspection (or after a cancellation is approved), to the same account or method you paid from.
-â€¢ To cancel or change a booking, message Flora Dress Rental Bohol on Facebook with your booking code.</t>
+• Refunds are sent within 3 business days after return and inspection (or after a cancellation is approved), to the same account or method you paid from.
+• To cancel or change a booking, message Flora Dress Rental Bohol on Facebook with your booking code.</t>
         </is>
       </c>
       <c r="C22" s="4" t="inlineStr">

</xml_diff>

<commit_message>
Prepare for public launch: no AI badges, hourly pickup, approved policies
- Remove "AI-styled preview" badges and alt text from cards, gallery and the
  reserve picker; a dress with no real photos shows one neutral line asking
  customers to message for real photos before booking.
- Pickup times hourly 8:00 AM-8:00 PM; privacy notice approved with 1-year
  retention; rental terms and cancellation policy approved as drafted.
- Publish all 11 dresses in the Sheet's starting catalog; preview mode uses
  the real terms and privacy notice.
- Rebuild the Sheet template; update docs and keep the catalog test fixture
  unpublished except its two test dresses.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/sheets-template/Flora_Booking_Sheet_Template.xlsx
+++ b/sheets-template/Flora_Booking_Sheet_Template.xlsx
@@ -543,7 +543,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Small</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -563,7 +563,7 @@
         <v>3</v>
       </c>
       <c r="N2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3">
@@ -604,7 +604,7 @@
         <v>3</v>
       </c>
       <c r="N3" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4">
@@ -623,6 +623,11 @@
           <t>Beige lace midi dress with thin straps, a boned straight neckline and a soft A-line skirt.</t>
         </is>
       </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Small</t>
+        </is>
+      </c>
       <c r="E4" t="inlineStr">
         <is>
           <t>Beige</t>
@@ -640,7 +645,7 @@
         <v>3</v>
       </c>
       <c r="N4" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5">
@@ -681,7 +686,7 @@
         <v>3</v>
       </c>
       <c r="N5" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6">
@@ -722,7 +727,7 @@
         <v>3</v>
       </c>
       <c r="N6" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7">
@@ -763,7 +768,7 @@
         <v>3</v>
       </c>
       <c r="N7" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="8">
@@ -804,7 +809,7 @@
         <v>3</v>
       </c>
       <c r="N8" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9">
@@ -845,7 +850,7 @@
         <v>3</v>
       </c>
       <c r="N9" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="10">
@@ -886,7 +891,7 @@
         <v>3</v>
       </c>
       <c r="N10" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="11">
@@ -927,7 +932,7 @@
         <v>3</v>
       </c>
       <c r="N11" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="12">
@@ -968,7 +973,7 @@
         <v>3</v>
       </c>
       <c r="N12" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="13">
@@ -13301,10 +13306,14 @@
           <t>operating_hours</t>
         </is>
       </c>
-      <c r="B5" s="3" t="n"/>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Mondayâ€“Sunday, 7:30 AMâ€“8:30 PM</t>
+        </is>
+      </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>REQUIRED. Example: "Daily, 10:00 AM â€“ 6:00 PM".</t>
+          <t>Owner-confirmed hours. Pickup slots and return deadline are separate settings.</t>
         </is>
       </c>
     </row>
@@ -13314,10 +13323,26 @@
           <t>pickup_time_slots</t>
         </is>
       </c>
-      <c r="B6" s="3" t="n"/>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>8:00 AM
+9:00 AM
+10:00 AM
+11:00 AM
+12:00 PM
+1:00 PM
+2:00 PM
+3:00 PM
+4:00 PM
+5:00 PM
+6:00 PM
+7:00 PM
+8:00 PM</t>
+        </is>
+      </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>REQUIRED. One time per line, e.g. 10:00 AM / 12:00 PM / 2:00 PM / 4:00 PM.</t>
+          <t>Owner-confirmed hourly pickup times (2026-10-24). One time per line.</t>
         </is>
       </c>
     </row>
@@ -13327,10 +13352,14 @@
           <t>return_deadline_time</t>
         </is>
       </c>
-      <c r="B7" s="3" t="n"/>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>8:30 PM</t>
+        </is>
+      </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>REQUIRED. Time the dress is due back on the return date, e.g. 6:00 PM.</t>
+          <t>Owner-confirmed deadline on the return date (Asia/Manila).</t>
         </is>
       </c>
     </row>
@@ -13582,10 +13611,20 @@
           <t>privacy_notice</t>
         </is>
       </c>
-      <c r="B21" s="3" t="n"/>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>FLORA DRESS RENTAL â€” PRIVACY NOTICE
+We collect your name, mobile number, Facebook profile name and booking details when you request a reservation. We use them only to review and manage your rental: verifying your request through Facebook, contacting you about payment, pickup and return, and keeping a record of the rental and deposit.
+We check your government-issued photo ID in person at pickup and do not keep a copy.
+Your details are stored in a private Google Sheet that only Flora staff can access. They are not sold or shared except where required by law.
+We keep booking records for 1 year after your rental is completed, for accounting and dispute purposes, then delete them.
+To ask what we hold, correct it, or request deletion, message our Facebook Page.
+This notice follows the Philippine Data Privacy Act of 2012 (RA 10173).</t>
+        </is>
+      </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
-          <t>REQUIRED. Paste the owner-approved privacy notice (a draft is in docs/OWNER_SETTINGS.md).</t>
+          <t>Owner-approved 2026-10-24 (1-year retention). Have someone with legal knowledge review it if possible.</t>
         </is>
       </c>
     </row>

</xml_diff>